<commit_message>
[ADD] ajuste para campo de embargos, y mejorar descripcion campo observaciones
</commit_message>
<xml_diff>
--- a/Plantilla_ALCANCE.xlsx
+++ b/Plantilla_ALCANCE.xlsx
@@ -1,10 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15FB6519-EA1B-46EB-A9B3-681A0D6C0E27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="ALCANCE" state="visible" r:id="rId4"/>
+    <sheet name="ALCANCE" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -217,18 +221,20 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -253,22 +259,44 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -607,33 +635,35 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:U4"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="23" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="19" customWidth="1"/>
-    <col min="7" max="7" width="50" customWidth="1"/>
-    <col min="8" max="8" width="34" customWidth="1"/>
-    <col min="9" max="9" width="55" customWidth="1"/>
-    <col min="10" max="10" width="22" customWidth="1"/>
-    <col min="11" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="21" customWidth="1"/>
-    <col min="13" max="13" width="20" customWidth="1"/>
-    <col min="14" max="14" width="21" customWidth="1"/>
-    <col min="15" max="15" width="30" customWidth="1"/>
-    <col min="16" max="16" width="18" customWidth="1"/>
-    <col min="17" max="17" width="24" customWidth="1"/>
-    <col min="18" max="18" width="35" customWidth="1"/>
-    <col min="19" max="19" width="36" customWidth="1"/>
-    <col min="20" max="20" width="25" customWidth="1"/>
-    <col min="21" max="21" width="18" customWidth="1"/>
+    <col min="1" max="1" width="18" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.21875" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.21875" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="48.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="32.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="42.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.21875" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="29.77734375" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="26.77734375" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="32.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="34.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="22.77734375" style="3" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="19.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="22" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -652,7 +682,7 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
@@ -698,203 +728,203 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="4">
         <v>5000000</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="G2" s="2">
+      <c r="G2" s="5">
         <v>110014189005</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="M2" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="N2" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="O2" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="P2" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="Q2" s="2" t="s">
+      <c r="Q2" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="R2" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="S2" s="2" t="s">
+      <c r="S2" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="T2" s="2" t="s">
+      <c r="T2" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="U2" s="2" t="s">
+      <c r="U2" s="4" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="4">
         <v>0</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="L3" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="M3" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="N3" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="O3" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="P3" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="Q3" s="2" t="s">
+      <c r="Q3" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="R3" s="2" t="s">
+      <c r="R3" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="S3" s="2" t="s">
+      <c r="S3" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="T3" s="2" t="s">
+      <c r="T3" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="U3" s="2" t="s">
+      <c r="U3" s="4" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="4">
         <v>2000000</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="5">
         <v>110014189007</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="J4" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="K4" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="L4" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="M4" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="N4" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="O4" s="2" t="s">
+      <c r="O4" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="P4" s="2" t="s">
+      <c r="P4" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="Q4" s="2" t="s">
+      <c r="Q4" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="R4" s="2" t="s">
+      <c r="R4" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="S4" s="2" t="s">
+      <c r="S4" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="T4" s="2" t="s">
+      <c r="T4" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="U4" s="2" t="s">
+      <c r="U4" s="4" t="s">
         <v>66</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>